<commit_message>
Add TP=2/TP=4 scaling + communication overhead analysis (report section 9)
- TP2/TP4 x bs1/bs64 profiling on PCIe-only RTX PRO 5000 node
- EP unsupported by b12x NVFP4 MoE kernel (ValueError) - TP allreduce only
- TP2 is sweet spot: decode b64 1.52x busy speedup, comm 8.3%; TP4 comm explodes to 44%
- bs1 multi-GPU is wall-clock negative; small payloads use fast b12x pcie_allreduce
- Excel: new TP overview + comm analysis sheets
</commit_message>
<xml_diff>
--- a/rtx6000d/results/DeepSeekV4_NVFP4_profiling_comparison.xlsx
+++ b/rtx6000d/results/DeepSeekV4_NVFP4_profiling_comparison.xlsx
@@ -11,6 +11,8 @@
     <sheet name="prefill breakdown" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="decode breakdown" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="NVFP4 分析" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TP扩展总览" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TP通信分析" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +51,11 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -62,11 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2062,9 +2070,6 @@
           <t>MoE routed experts w1/w2/w3 GEMM + SiLU 融合 (唯一 NVFP4 算子)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2077,9 +2082,6 @@
           <t>88.8% (145.1/163.5 GiB)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2092,9 +2094,6 @@
           <t>~51%</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2107,9 +2106,1210 @@
           <t>57 vs 100 vs 201 MB/层</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>GPU busy (ms)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>vs TP1 加速比</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>wall (ms)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>wall vs TP1</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>吞吐 tok/s (wall)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>通信 (ms)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>通信占 busy</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>MoE NVFP4 (ms)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>MoE 占 busy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>291</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>56.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="H3" t="n">
+        <v>267</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>43.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="F4" t="n">
+        <v>59</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="H4" t="n">
+        <v>271</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>36.2%</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>30.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>32.28</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>360</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2844</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>20.61</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>63.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>64</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F6" t="n">
+        <v>256</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>53.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>64</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>27.31</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F7" t="n">
+        <v>255</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4016</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>14.78</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>54.1%</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>22.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>73</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>219</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>13.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>20.17</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="H9" t="n">
+        <v>200</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>24.2%</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F10" t="n">
+        <v>82</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="H10" t="n">
+        <v>195</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>64</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>133.34</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>220</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4655</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>63.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>64</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>87.61</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F12" t="n">
+        <v>182</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5626</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>45.35</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>51.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>64</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>99.43000000000001</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F13" t="n">
+        <v>207</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4947</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>43.96</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>44.2%</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>26.9%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>NCCL AllReduce ms(calls)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NCCL AllGather ms(calls)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>b12x PCIe-AR ms(calls)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>通信合计 ms</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>通信占 busy</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>单次 AllReduce 均值 us</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.40(5)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.01(1)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.64(5)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.02(1)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>36.2%</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>127.3</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>64</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1.27(15)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.29(3)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>64</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>12.29(15)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2.50(3)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>14.78</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>54.1%</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>819.1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>prefill 每步 AR payload 大(1024 tok),54% busy 是通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.42(16)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>4.45(80)</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>24.2%</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.24(16)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1.25(80)</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>小 payload 走 b12x pcie_allreduce(80 次,~15.6us/次)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>64</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>64</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2.87(130)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>4.36(28)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.05(10)</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>AllReduce 为主;MoE expert 按 TP 切半</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>64</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>22.35(145)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>7.29(32)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>14.32(15)</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>43.96</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>44.2%</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>154.1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>NCCL AR 22.4ms + PCIe-AR 14.3ms 双路径;PCIe ring 是瓶颈</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add TP2+EP (marlin) profiling: EP communication pattern实测对比
- Root cause: b12x MoE kernel hard-rejects EP (b12x_moe.py _supports_parallel_config);
  swiglu_limit oracle gate blocks all alternative NVFP4 backends except trtllm (no sm120)
- Patched oracle clamp gate: marlin backend loads with --enable-expert-parallel (W4A16, no FP4 TC, no clamp)
- EP comm is NOT all2all: AllGather dispatch + full-hidden AllReduce combine; comm 45-82% of busy vs TP2 8.3%
- decode b64: EP busy 143ms vs TP2 88ms (1.6x GPU cost/token); prefill b64 AR avg 4.59ms/call, 82% busy
- Conclusion: EP not viable on this stack + PCIe topology; TP=2 remains the cap
- Excel: new EP对比 sheet; report section 9.5 + revised 9.1/9.4
</commit_message>
<xml_diff>
--- a/rtx6000d/results/DeepSeekV4_NVFP4_profiling_comparison.xlsx
+++ b/rtx6000d/results/DeepSeekV4_NVFP4_profiling_comparison.xlsx
@@ -13,6 +13,7 @@
     <sheet name="NVFP4 分析" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="TP扩展总览" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="TP通信分析" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="EP对比" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2843,7 +2844,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2883,7 +2883,6 @@
       <c r="I3" s="4" t="n">
         <v>79.7</v>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2923,7 +2922,6 @@
       <c r="I4" s="4" t="n">
         <v>127.3</v>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2965,7 +2963,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3005,7 +3002,6 @@
       <c r="I6" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3091,7 +3087,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3133,7 +3128,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3221,7 +3215,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3308,6 +3301,542 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>NCCL AR 22.4ms + PCIe-AR 14.3ms 双路径;PCIe ring 是瓶颈</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>GPU busy (ms)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>wall (ms)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>通信 (ms)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>通信占 busy</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>MoE (ms)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>MoE kernel</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>AR ms(calls)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>AG ms(calls)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>PCIe-AR ms(calls)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TP2 (b12x MoE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="E2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>b12x fused NVFP4</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.40(5)</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.01(1)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TP2+EP (marlin MoE)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="E3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>marlin W4A16 (dequant+bf16)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.15(5)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.01(1)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>marlin W4A16 MoE;小流量通信少</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>64</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TP2 (b12x MoE)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="E4" t="n">
+        <v>256</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>b12x fused NVFP4</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1.27(15)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.29(3)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>prefill</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TP2+EP (marlin MoE)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>89.81</v>
+      </c>
+      <c r="E5" t="n">
+        <v>240</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>73.63</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>82.0%</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>marlin W4A16 (dequant+bf16)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>68.87(15)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>4.76(3)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>NCCL AR 均 4.59ms/次,通信 82% busy;dispatch 走 AllGather(非 AllToAll)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TP2 (b12x MoE)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>20.17</v>
+      </c>
+      <c r="E6" t="n">
+        <v>80</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>24.2%</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>b12x fused NVFP4</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0.42(16)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>4.45(80)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TP2+EP (marlin MoE)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="E7" t="n">
+        <v>77</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>40.01</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>71.5%</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>marlin W4A16 (dequant+bf16)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0.00(0)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0.47(16)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>39.54(80)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>PCIe-AR 均 494us/次(vs TP2 15.6us)——EP 合并全量 hidden 输出,AR payload 不随 rank 缩小</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>64</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TP2 (b12x MoE)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>87.61</v>
+      </c>
+      <c r="E8" t="n">
+        <v>182</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>45.35</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>b12x fused NVFP4</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2.87(130)</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>4.36(28)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.05(10)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>decode</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>64</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TP2+EP (marlin MoE)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>143.28</v>
+      </c>
+      <c r="E9" t="n">
+        <v>175</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>65.19</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>45.5%</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>42.43</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>marlin W4A16 (dequant+bf16)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>37.46(115)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>6.61(26)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>21.12(15)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>marlin MoE 42.4ms 与 b12x 45.4ms 相当,但通信 65.2ms(45.5%)远高于 TP2 的 8.3%</t>
         </is>
       </c>
     </row>

</xml_diff>